<commit_message>
actualiza acumulados 25/06/2026 17:40
</commit_message>
<xml_diff>
--- a/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO LUIS LOPEZ DE MESA IED-502_Ajustado_20260625_155744.xlsx
+++ b/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO LUIS LOPEZ DE MESA IED-502_Ajustado_20260625_155744.xlsx
@@ -5,22 +5,29 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\Ajustar 3 y 5\Ajustados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\PRUEBAS A CALIFICAR\Ya procesadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_BB925F48915EE44F6B74DC97565DCE3A97C528E5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C96C93E8-2EED-42F7-8465-444B3A7CB518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="720" windowWidth="19190" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
+    <sheet name="Resultados" sheetId="1" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Resultados!$A$1:$AB$77</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
+  <pivotCaches>
+    <pivotCache cacheId="23" r:id="rId3"/>
+  </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2009" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2051" uniqueCount="118">
   <si>
     <t>Est.</t>
   </si>
@@ -362,6 +369,18 @@
   </si>
   <si>
     <t>1023407027</t>
+  </si>
+  <si>
+    <t>Etiquetas de fila</t>
+  </si>
+  <si>
+    <t>(en blanco)</t>
+  </si>
+  <si>
+    <t>Total general</t>
+  </si>
+  <si>
+    <t>Cuenta de Cód.Est.</t>
   </si>
 </sst>
 </file>
@@ -415,12 +434,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,6 +460,2679 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Catherine Espinosa Perez" refreshedDate="46198.67199722222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="77" xr:uid="{E0318AEC-D8E7-492E-AE59-D6367915CC04}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:AB1048576" sheet="Resultados"/>
+  </cacheSource>
+  <cacheFields count="28">
+    <cacheField name="Est." numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="39"/>
+    </cacheField>
+    <cacheField name="Cód.Sede" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Nombre Sede" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Estudiante" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Cód.Est." numFmtId="0">
+      <sharedItems containsBlank="1" count="39">
+        <s v="1012433627"/>
+        <s v="1146136808"/>
+        <s v="7312317"/>
+        <s v="1012448808"/>
+        <s v="1011238803"/>
+        <s v="1121717186"/>
+        <s v="1021408881"/>
+        <s v="1012454385"/>
+        <s v="1012452067"/>
+        <s v="1070979655"/>
+        <s v="1030679820"/>
+        <s v="1028791681"/>
+        <s v="1233492864"/>
+        <s v="1146136686"/>
+        <s v="1141350561"/>
+        <s v="1146132578"/>
+        <s v="1031844011"/>
+        <s v="1024582657"/>
+        <s v="1111583961"/>
+        <s v="1037502564"/>
+        <s v="1146133728"/>
+        <s v="1011241134"/>
+        <s v="1073706266"/>
+        <s v="1012447184"/>
+        <s v="1146137513"/>
+        <s v="N37664898212"/>
+        <s v="1028791887"/>
+        <s v="1146135454"/>
+        <s v="1025557079"/>
+        <s v="1012444181"/>
+        <s v="1012449656"/>
+        <s v="1012449779"/>
+        <s v="1079233445"/>
+        <s v="1012445431"/>
+        <s v="1030655365"/>
+        <s v="N37646730296"/>
+        <s v="5300568"/>
+        <s v="1023407027"/>
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Grado" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Grupo" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Materia" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P01" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P02" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P03" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P04" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P05" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P06" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P07" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P08" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P09" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P10" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P11" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P12" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P13" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P14" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P15" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P16" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P17" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P18" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P19" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="P20" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="77">
+  <r>
+    <n v="1"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SAMUEL MATIAS VENEGAS MORENO"/>
+    <x v="0"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="1"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SAMUEL MATIAS VENEGAS MORENO"/>
+    <x v="0"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="2"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SARA LUCIANA ROMERO SIMBAQUEBA"/>
+    <x v="1"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="2"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SARA LUCIANA ROMERO SIMBAQUEBA"/>
+    <x v="1"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="3"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="WUILMARY CONSOLACION BOHORQUEZ HERRERA"/>
+    <x v="2"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="3"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="WUILMARY CONSOLACION BOHORQUEZ HERRERA"/>
+    <x v="2"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <m/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="4"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN DIEGO ESCOBAR PAJARITO"/>
+    <x v="3"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="C"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="4"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN DIEGO ESCOBAR PAJARITO"/>
+    <x v="3"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="5"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="GERMAN ESTEBAN AMORTEGUI FERNANDEZ"/>
+    <x v="4"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <n v="5"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="GERMAN ESTEBAN AMORTEGUI FERNANDEZ"/>
+    <x v="4"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="TANIA YULIANA PEREZ VELASQUEZ"/>
+    <x v="5"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="TANIA YULIANA PEREZ VELASQUEZ"/>
+    <x v="5"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="7"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SAMUEL FELIPE PACHECO MARTINEZ"/>
+    <x v="6"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="7"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SAMUEL FELIPE PACHECO MARTINEZ"/>
+    <x v="6"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="8"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="EMILY SOFIA ORTIZ CORREA"/>
+    <x v="7"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="8"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="EMILY SOFIA ORTIZ CORREA"/>
+    <x v="7"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="9"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MIA ISABELLA LOPEZ ORTIZ"/>
+    <x v="8"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="9"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MIA ISABELLA LOPEZ ORTIZ"/>
+    <x v="8"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="10"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="AYLIN GABRIELA GALLO DIAZ"/>
+    <x v="9"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="10"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="AYLIN GABRIELA GALLO DIAZ"/>
+    <x v="9"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="11"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DAVIAN RANGEL MONTOYA"/>
+    <x v="10"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <n v="11"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DAVIAN RANGEL MONTOYA"/>
+    <x v="10"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="12"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="VALERIE SARAY MELO PULIDO"/>
+    <x v="11"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="12"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="VALERIE SARAY MELO PULIDO"/>
+    <x v="11"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="LEIDY SOFIA MORENO CARDONA"/>
+    <x v="12"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="LEIDY SOFIA MORENO CARDONA"/>
+    <x v="12"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <m/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="15"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="HELLEN SAMANTHA RUIZ OSORIO"/>
+    <x v="13"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="15"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="HELLEN SAMANTHA RUIZ OSORIO"/>
+    <x v="13"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="16"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="LORENZO ESTEBAN CARRANZA CORTES"/>
+    <x v="14"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="16"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="LORENZO ESTEBAN CARRANZA CORTES"/>
+    <x v="14"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <m/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <m/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="17"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN ANDRES ESQUIVEL PULIDO"/>
+    <x v="15"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="17"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN ANDRES ESQUIVEL PULIDO"/>
+    <x v="15"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="18"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SHERIL JOHANNA CUELLAR MARTINEZ"/>
+    <x v="16"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <m/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="18"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SHERIL JOHANNA CUELLAR MARTINEZ"/>
+    <x v="16"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="19"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ANA VICTORIA ROJAS MOLINA"/>
+    <x v="17"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <m/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="19"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ANA VICTORIA ROJAS MOLINA"/>
+    <x v="17"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <m/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="20"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="EDUBER GARCIA GUALDRON"/>
+    <x v="18"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="20"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="EDUBER GARCIA GUALDRON"/>
+    <x v="18"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="21"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MAXIMILIANO FRANCO SEPULVEDA"/>
+    <x v="19"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <m/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="21"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MAXIMILIANO FRANCO SEPULVEDA"/>
+    <x v="19"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="22"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SARA VALENTINA HERNANDEZ YATE"/>
+    <x v="20"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="22"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SARA VALENTINA HERNANDEZ YATE"/>
+    <x v="20"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="23"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="NOAH ISABELLA ALVAREZ MURCIA"/>
+    <x v="21"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="23"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="NOAH ISABELLA ALVAREZ MURCIA"/>
+    <x v="21"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <n v="24"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ALAN SANTIAGO VANEGAS"/>
+    <x v="22"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="24"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ALAN SANTIAGO VANEGAS"/>
+    <x v="22"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="25"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ANGUIE TATIANA SIERRA MARTIN"/>
+    <x v="23"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="25"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ANGUIE TATIANA SIERRA MARTIN"/>
+    <x v="23"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <n v="26"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="THOMAS MATEO MONTOYA RUIZ"/>
+    <x v="24"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="26"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="THOMAS MATEO MONTOYA RUIZ"/>
+    <x v="24"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="27"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DANIELYS STEPHANIA ROMERO ORTIZ"/>
+    <x v="25"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="27"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DANIELYS STEPHANIA ROMERO ORTIZ"/>
+    <x v="25"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="D"/>
+    <s v="D"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <n v="28"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN PABLO BOLIVAR GONZALEZ"/>
+    <x v="26"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <m/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="28"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN PABLO BOLIVAR GONZALEZ"/>
+    <x v="26"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <m/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <m/>
+  </r>
+  <r>
+    <n v="29"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MADELIN LUCIA GUTIERREZ RODRIGUEZ"/>
+    <x v="27"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <m/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="29"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MADELIN LUCIA GUTIERREZ RODRIGUEZ"/>
+    <x v="27"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="30"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="LIAN ARMANDO OQUENDO RODRIGUEZ"/>
+    <x v="28"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="30"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="LIAN ARMANDO OQUENDO RODRIGUEZ"/>
+    <x v="28"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="31"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DANNA YULITZA ROMERO MARIÑO"/>
+    <x v="29"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="31"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DANNA YULITZA ROMERO MARIÑO"/>
+    <x v="29"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="32"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="BREINER SEBASTIAN OTALORA GOMEZ"/>
+    <x v="30"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="32"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="BREINER SEBASTIAN OTALORA GOMEZ"/>
+    <x v="30"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="33"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ANGEL DANIEL LOAIZA CASTAÑEDA"/>
+    <x v="31"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="33"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ANGEL DANIEL LOAIZA CASTAÑEDA"/>
+    <x v="31"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="34"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="IAN SANTIAGO BELLO CASTILLO"/>
+    <x v="32"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="34"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="IAN SANTIAGO BELLO CASTILLO"/>
+    <x v="32"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="35"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN SEBASTIAN BUITRAGO GUARDIA"/>
+    <x v="33"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="35"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="JUAN SEBASTIAN BUITRAGO GUARDIA"/>
+    <x v="33"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="36"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MARIA ISABELLA BELTRAN TOVAR"/>
+    <x v="34"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+  </r>
+  <r>
+    <n v="36"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="MARIA ISABELLA BELTRAN TOVAR"/>
+    <x v="34"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+  </r>
+  <r>
+    <n v="37"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ARANZA NATALY LOPEZ RENGEL"/>
+    <x v="35"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="37"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="ARANZA NATALY LOPEZ RENGEL"/>
+    <x v="35"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="38"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SANTIAGO JOSE BORDONES POLANCO"/>
+    <x v="36"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="A"/>
+  </r>
+  <r>
+    <n v="38"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="SANTIAGO JOSE BORDONES POLANCO"/>
+    <x v="36"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <s v="C"/>
+    <s v="D"/>
+    <s v="A"/>
+    <m/>
+    <s v="A"/>
+    <s v="C"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="B"/>
+    <s v="C"/>
+    <s v="B"/>
+    <s v="D"/>
+    <s v="A"/>
+    <s v="A"/>
+    <s v="D"/>
+    <s v="C"/>
+    <s v="C"/>
+  </r>
+  <r>
+    <n v="39"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DANIEL ESCOBAR TRIANA"/>
+    <x v="37"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Matemáticas"/>
+    <s v="C"/>
+    <s v="C"/>
+    <s v="C"/>
+    <m/>
+    <s v="B"/>
+    <s v="B"/>
+    <s v="D"/>
+    <m/>
+    <m/>
+    <s v="C"/>
+    <s v="D"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <n v="39"/>
+    <s v="111102000265"/>
+    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
+    <s v="DANIEL ESCOBAR TRIANA"/>
+    <x v="37"/>
+    <s v="5"/>
+    <s v="0502"/>
+    <s v="Lenguaje"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <x v="38"/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EFFFE35C-FE5C-4BA9-BF73-424097ED36A7}" name="TablaDinámica5" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B43" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="28">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="40">
+        <item x="4"/>
+        <item x="21"/>
+        <item x="0"/>
+        <item x="29"/>
+        <item x="33"/>
+        <item x="23"/>
+        <item x="3"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="8"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="37"/>
+        <item x="17"/>
+        <item x="28"/>
+        <item x="11"/>
+        <item x="26"/>
+        <item x="34"/>
+        <item x="10"/>
+        <item x="16"/>
+        <item x="19"/>
+        <item x="9"/>
+        <item x="22"/>
+        <item x="32"/>
+        <item x="18"/>
+        <item x="5"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="20"/>
+        <item x="27"/>
+        <item x="13"/>
+        <item x="1"/>
+        <item x="24"/>
+        <item x="12"/>
+        <item x="36"/>
+        <item x="2"/>
+        <item x="35"/>
+        <item x="25"/>
+        <item x="38"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="40">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="35"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i>
+      <x v="38"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Cuenta de Cód.Est." fld="4" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -722,6 +3419,346 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB41E6A-960B-4B42-A92B-B9D287BB9BF0}">
+  <dimension ref="A3:B43"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B14" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B16" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B20" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B21" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B26" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B37" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B38" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B39" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B40" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B41" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B42" s="5"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B43" s="5">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7217,6 +10254,7 @@
       <c r="AB77" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AB77" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
actualiza acumulados 25/06/2026 19:16
</commit_message>
<xml_diff>
--- a/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO LUIS LOPEZ DE MESA IED-502_Ajustado_20260625_155744.xlsx
+++ b/PRUEBAS A CALIFICAR/Ya procesadas/COLEGIO LUIS LOPEZ DE MESA IED-502_Ajustado_20260625_155744.xlsx
@@ -8,26 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Espinosa\Desktop\PROYECTO JULIANA\PRUEBAS A CALIFICAR\Ya procesadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C96C93E8-2EED-42F7-8465-444B3A7CB518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A3A3F16-45F2-4D18-B25A-7FACEF9E3BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
-    <sheet name="Resultados" sheetId="1" r:id="rId2"/>
+    <sheet name="Resultados" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Resultados!$A$1:$AB$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Resultados!$A$1:$AB$77</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
-  <pivotCaches>
-    <pivotCache cacheId="23" r:id="rId3"/>
-  </pivotCaches>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2051" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2009" uniqueCount="114">
   <si>
     <t>Est.</t>
   </si>
@@ -369,18 +378,6 @@
   </si>
   <si>
     <t>1023407027</t>
-  </si>
-  <si>
-    <t>Etiquetas de fila</t>
-  </si>
-  <si>
-    <t>(en blanco)</t>
-  </si>
-  <si>
-    <t>Total general</t>
-  </si>
-  <si>
-    <t>Cuenta de Cód.Est.</t>
   </si>
 </sst>
 </file>
@@ -434,17 +431,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,2679 +452,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Catherine Espinosa Perez" refreshedDate="46198.67199722222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="77" xr:uid="{E0318AEC-D8E7-492E-AE59-D6367915CC04}">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A1:AB1048576" sheet="Resultados"/>
-  </cacheSource>
-  <cacheFields count="28">
-    <cacheField name="Est." numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="1" maxValue="39"/>
-    </cacheField>
-    <cacheField name="Cód.Sede" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Nombre Sede" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Estudiante" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Cód.Est." numFmtId="0">
-      <sharedItems containsBlank="1" count="39">
-        <s v="1012433627"/>
-        <s v="1146136808"/>
-        <s v="7312317"/>
-        <s v="1012448808"/>
-        <s v="1011238803"/>
-        <s v="1121717186"/>
-        <s v="1021408881"/>
-        <s v="1012454385"/>
-        <s v="1012452067"/>
-        <s v="1070979655"/>
-        <s v="1030679820"/>
-        <s v="1028791681"/>
-        <s v="1233492864"/>
-        <s v="1146136686"/>
-        <s v="1141350561"/>
-        <s v="1146132578"/>
-        <s v="1031844011"/>
-        <s v="1024582657"/>
-        <s v="1111583961"/>
-        <s v="1037502564"/>
-        <s v="1146133728"/>
-        <s v="1011241134"/>
-        <s v="1073706266"/>
-        <s v="1012447184"/>
-        <s v="1146137513"/>
-        <s v="N37664898212"/>
-        <s v="1028791887"/>
-        <s v="1146135454"/>
-        <s v="1025557079"/>
-        <s v="1012444181"/>
-        <s v="1012449656"/>
-        <s v="1012449779"/>
-        <s v="1079233445"/>
-        <s v="1012445431"/>
-        <s v="1030655365"/>
-        <s v="N37646730296"/>
-        <s v="5300568"/>
-        <s v="1023407027"/>
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Grado" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Grupo" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Materia" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P01" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P02" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P03" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P04" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P05" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P06" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P07" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P08" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P09" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P10" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P11" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P12" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P13" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P14" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P15" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P16" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P17" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P18" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P19" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-    <cacheField name="P20" numFmtId="0">
-      <sharedItems containsBlank="1"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="77">
-  <r>
-    <n v="1"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SAMUEL MATIAS VENEGAS MORENO"/>
-    <x v="0"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="1"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SAMUEL MATIAS VENEGAS MORENO"/>
-    <x v="0"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SARA LUCIANA ROMERO SIMBAQUEBA"/>
-    <x v="1"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SARA LUCIANA ROMERO SIMBAQUEBA"/>
-    <x v="1"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="WUILMARY CONSOLACION BOHORQUEZ HERRERA"/>
-    <x v="2"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="WUILMARY CONSOLACION BOHORQUEZ HERRERA"/>
-    <x v="2"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <m/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN DIEGO ESCOBAR PAJARITO"/>
-    <x v="3"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <m/>
-    <m/>
-    <m/>
-    <s v="C"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN DIEGO ESCOBAR PAJARITO"/>
-    <x v="3"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="GERMAN ESTEBAN AMORTEGUI FERNANDEZ"/>
-    <x v="4"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <n v="5"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="GERMAN ESTEBAN AMORTEGUI FERNANDEZ"/>
-    <x v="4"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="TANIA YULIANA PEREZ VELASQUEZ"/>
-    <x v="5"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="B"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="TANIA YULIANA PEREZ VELASQUEZ"/>
-    <x v="5"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SAMUEL FELIPE PACHECO MARTINEZ"/>
-    <x v="6"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SAMUEL FELIPE PACHECO MARTINEZ"/>
-    <x v="6"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="EMILY SOFIA ORTIZ CORREA"/>
-    <x v="7"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="EMILY SOFIA ORTIZ CORREA"/>
-    <x v="7"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MIA ISABELLA LOPEZ ORTIZ"/>
-    <x v="8"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MIA ISABELLA LOPEZ ORTIZ"/>
-    <x v="8"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="AYLIN GABRIELA GALLO DIAZ"/>
-    <x v="9"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="AYLIN GABRIELA GALLO DIAZ"/>
-    <x v="9"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="11"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DAVIAN RANGEL MONTOYA"/>
-    <x v="10"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-  </r>
-  <r>
-    <n v="11"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DAVIAN RANGEL MONTOYA"/>
-    <x v="10"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="12"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="VALERIE SARAY MELO PULIDO"/>
-    <x v="11"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="12"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="VALERIE SARAY MELO PULIDO"/>
-    <x v="11"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="14"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="LEIDY SOFIA MORENO CARDONA"/>
-    <x v="12"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="14"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="LEIDY SOFIA MORENO CARDONA"/>
-    <x v="12"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <m/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="15"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="HELLEN SAMANTHA RUIZ OSORIO"/>
-    <x v="13"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="15"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="HELLEN SAMANTHA RUIZ OSORIO"/>
-    <x v="13"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="16"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="LORENZO ESTEBAN CARRANZA CORTES"/>
-    <x v="14"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="16"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="LORENZO ESTEBAN CARRANZA CORTES"/>
-    <x v="14"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <m/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <m/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="17"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN ANDRES ESQUIVEL PULIDO"/>
-    <x v="15"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="17"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN ANDRES ESQUIVEL PULIDO"/>
-    <x v="15"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="18"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SHERIL JOHANNA CUELLAR MARTINEZ"/>
-    <x v="16"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <m/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="18"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SHERIL JOHANNA CUELLAR MARTINEZ"/>
-    <x v="16"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="19"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ANA VICTORIA ROJAS MOLINA"/>
-    <x v="17"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <m/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="19"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ANA VICTORIA ROJAS MOLINA"/>
-    <x v="17"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <m/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="20"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="EDUBER GARCIA GUALDRON"/>
-    <x v="18"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="20"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="EDUBER GARCIA GUALDRON"/>
-    <x v="18"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="21"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MAXIMILIANO FRANCO SEPULVEDA"/>
-    <x v="19"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <m/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="21"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MAXIMILIANO FRANCO SEPULVEDA"/>
-    <x v="19"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="22"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SARA VALENTINA HERNANDEZ YATE"/>
-    <x v="20"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="22"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SARA VALENTINA HERNANDEZ YATE"/>
-    <x v="20"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="23"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="NOAH ISABELLA ALVAREZ MURCIA"/>
-    <x v="21"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="23"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="NOAH ISABELLA ALVAREZ MURCIA"/>
-    <x v="21"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-  </r>
-  <r>
-    <n v="24"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ALAN SANTIAGO VANEGAS"/>
-    <x v="22"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="24"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ALAN SANTIAGO VANEGAS"/>
-    <x v="22"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="25"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ANGUIE TATIANA SIERRA MARTIN"/>
-    <x v="23"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="25"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ANGUIE TATIANA SIERRA MARTIN"/>
-    <x v="23"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-  </r>
-  <r>
-    <n v="26"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="THOMAS MATEO MONTOYA RUIZ"/>
-    <x v="24"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="26"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="THOMAS MATEO MONTOYA RUIZ"/>
-    <x v="24"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="27"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DANIELYS STEPHANIA ROMERO ORTIZ"/>
-    <x v="25"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="27"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DANIELYS STEPHANIA ROMERO ORTIZ"/>
-    <x v="25"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="D"/>
-    <s v="D"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-  </r>
-  <r>
-    <n v="28"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN PABLO BOLIVAR GONZALEZ"/>
-    <x v="26"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <m/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="28"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN PABLO BOLIVAR GONZALEZ"/>
-    <x v="26"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <m/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <m/>
-  </r>
-  <r>
-    <n v="29"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MADELIN LUCIA GUTIERREZ RODRIGUEZ"/>
-    <x v="27"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <m/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="29"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MADELIN LUCIA GUTIERREZ RODRIGUEZ"/>
-    <x v="27"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="30"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="LIAN ARMANDO OQUENDO RODRIGUEZ"/>
-    <x v="28"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="30"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="LIAN ARMANDO OQUENDO RODRIGUEZ"/>
-    <x v="28"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="31"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DANNA YULITZA ROMERO MARIÑO"/>
-    <x v="29"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="31"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DANNA YULITZA ROMERO MARIÑO"/>
-    <x v="29"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="32"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="BREINER SEBASTIAN OTALORA GOMEZ"/>
-    <x v="30"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="32"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="BREINER SEBASTIAN OTALORA GOMEZ"/>
-    <x v="30"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="33"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ANGEL DANIEL LOAIZA CASTAÑEDA"/>
-    <x v="31"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="33"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ANGEL DANIEL LOAIZA CASTAÑEDA"/>
-    <x v="31"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="34"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="IAN SANTIAGO BELLO CASTILLO"/>
-    <x v="32"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="34"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="IAN SANTIAGO BELLO CASTILLO"/>
-    <x v="32"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="35"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN SEBASTIAN BUITRAGO GUARDIA"/>
-    <x v="33"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="35"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="JUAN SEBASTIAN BUITRAGO GUARDIA"/>
-    <x v="33"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="36"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MARIA ISABELLA BELTRAN TOVAR"/>
-    <x v="34"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-  </r>
-  <r>
-    <n v="36"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="MARIA ISABELLA BELTRAN TOVAR"/>
-    <x v="34"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-  </r>
-  <r>
-    <n v="37"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ARANZA NATALY LOPEZ RENGEL"/>
-    <x v="35"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="37"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="ARANZA NATALY LOPEZ RENGEL"/>
-    <x v="35"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="38"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SANTIAGO JOSE BORDONES POLANCO"/>
-    <x v="36"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="A"/>
-  </r>
-  <r>
-    <n v="38"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="SANTIAGO JOSE BORDONES POLANCO"/>
-    <x v="36"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <s v="C"/>
-    <s v="D"/>
-    <s v="A"/>
-    <m/>
-    <s v="A"/>
-    <s v="C"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="B"/>
-    <s v="C"/>
-    <s v="B"/>
-    <s v="D"/>
-    <s v="A"/>
-    <s v="A"/>
-    <s v="D"/>
-    <s v="C"/>
-    <s v="C"/>
-  </r>
-  <r>
-    <n v="39"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DANIEL ESCOBAR TRIANA"/>
-    <x v="37"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Matemáticas"/>
-    <s v="C"/>
-    <s v="C"/>
-    <s v="C"/>
-    <m/>
-    <s v="B"/>
-    <s v="B"/>
-    <s v="D"/>
-    <m/>
-    <m/>
-    <s v="C"/>
-    <s v="D"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <n v="39"/>
-    <s v="111102000265"/>
-    <s v="COLEGIO LUIS LOPEZ DE MESA (IED)"/>
-    <s v="DANIEL ESCOBAR TRIANA"/>
-    <x v="37"/>
-    <s v="5"/>
-    <s v="0502"/>
-    <s v="Lenguaje"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="38"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-</pivotCacheRecords>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EFFFE35C-FE5C-4BA9-BF73-424097ED36A7}" name="TablaDinámica5" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:B43" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="28">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="40">
-        <item x="4"/>
-        <item x="21"/>
-        <item x="0"/>
-        <item x="29"/>
-        <item x="33"/>
-        <item x="23"/>
-        <item x="3"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="8"/>
-        <item x="7"/>
-        <item x="6"/>
-        <item x="37"/>
-        <item x="17"/>
-        <item x="28"/>
-        <item x="11"/>
-        <item x="26"/>
-        <item x="34"/>
-        <item x="10"/>
-        <item x="16"/>
-        <item x="19"/>
-        <item x="9"/>
-        <item x="22"/>
-        <item x="32"/>
-        <item x="18"/>
-        <item x="5"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="20"/>
-        <item x="27"/>
-        <item x="13"/>
-        <item x="1"/>
-        <item x="24"/>
-        <item x="12"/>
-        <item x="36"/>
-        <item x="2"/>
-        <item x="35"/>
-        <item x="25"/>
-        <item x="38"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="40">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="30"/>
-    </i>
-    <i>
-      <x v="31"/>
-    </i>
-    <i>
-      <x v="32"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i>
-      <x v="34"/>
-    </i>
-    <i>
-      <x v="35"/>
-    </i>
-    <i>
-      <x v="36"/>
-    </i>
-    <i>
-      <x v="37"/>
-    </i>
-    <i>
-      <x v="38"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Cuenta de Cód.Est." fld="4" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3419,346 +738,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB41E6A-960B-4B42-A92B-B9D287BB9BF0}">
-  <dimension ref="A3:B43"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="16.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B7" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B11" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B12" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B14" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B16" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B17" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B18" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B20" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B21" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B22" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B24" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B25" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B26" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B27" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B28" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B30" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B31" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B32" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B33" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B34" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B37" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B38" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B39" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B40" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B41" s="5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B42" s="5"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B43" s="5">
-        <v>76</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>